<commit_message>
Planilha: não perder quem bancou nem quem leva o prêmio
Duas coisas se perdiam calado na ponte com a planilha, as duas na parte de
sociedade entre arrematantes:

- O sócio escolhido para levar o prêmio inteiro (a.recebedor) não tinha
  coluna nenhuma. Quem marcasse a escolha no site, exportasse e importasse
  de volta via o prêmio voltar rachado entre os sócios — dinheiro diferente,
  sem aviso. Agora a coluna QUEM LEVA aceita o nome de um sócio, além de
  cotas / pagador como antes, e um nome que não seja de sócio gera aviso em
  vez de sumir.
- Na coluna PAGOU da aba Socios, "sim" quer dizer "pagou a própria cota".
  Quem escrevesse "sim" para o sócio que bancou o lance inteiro ficava com
  metade do lance em aberto no clube. Agora "bancou tudo" (ou "tudo",
  "integral") vale o lance inteiro, e as instruções do modelo explicam a
  diferença.

O exemplo da aba Socios no modelo passa a usar "bancou tudo", e um teste
importa o próprio modelo para garantir que o exemplo fecha a conta.
</commit_message>
<xml_diff>
--- a/modelo-planilha-apostas.xlsx
+++ b/modelo-planilha-apostas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A37"/>
   <cols>
     <col min="1" max="1" width="78.83203125" customWidth="1"/>
   </cols>
@@ -468,92 +468,107 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">  PAGOU       quanto essa pessoa pôs do próprio bolso (pode ser zero).</v>
+        <v xml:space="preserve">  PAGOU       quanto essa pessoa pôs do próprio bolso, em reais (pode</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  QUEM LEVA   cotas (cada sócio recebe a parte dele, já descontando o</v>
+        <v xml:space="preserve">              ser zero). Vale escrever bancou tudo quando ela pagou o</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">              que devia) ou pagador (o prêmio inteiro vai para quem</v>
+        <v xml:space="preserve">              lance inteiro. Um sim aqui quer dizer só a própria cota.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">              bancou o lance, e os sócios acertam por fora).</v>
+        <v xml:space="preserve">  QUEM LEVA   cotas (cada sócio recebe a parte dele, já descontando o</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">  A competição e o atirador repetem a linha de cima se ficarem em branco.</v>
+        <v xml:space="preserve">              que devia), pagador (o prêmio inteiro vai para quem</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v xml:space="preserve">              bancou o lance, e os sócios acertam por fora), ou o nome</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Na aba RESULTADO, informe o pódio e quanto vale cada colocação.</v>
+        <v xml:space="preserve">              de um sócio, para o prêmio ir todo para ele.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  COLOCACAO   1, 2, 3… quantas o clube premiar.</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v xml:space="preserve">  PERCENTUAL  quanto do bolo vai para aquela colocação (50, 30, 20…).</v>
+        <v xml:space="preserve">  A competição e o atirador repetem a linha de cima se ficarem em branco.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  Pode acrescentar linhas para 4º, 5º lugar — ou usar só 1º e 2º.</v>
+        <v>Na aba RESULTADO, informe o pódio e quanto vale cada colocação.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  Os percentuais não precisam somar 100: o bolo é dividido na proporção.</v>
+        <v xml:space="preserve">  COLOCACAO   1, 2, 3… quantas o clube premiar.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v xml:space="preserve">  PERCENTUAL  quanto do bolo vai para aquela colocação (50, 30, 20…).</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>A aba AJUSTES é opcional:</v>
+        <v xml:space="preserve">  Pode acrescentar linhas para 4º, 5º lugar — ou usar só 1º e 2º.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  RATEIO  proporcional (quem apostou mais leva mais) ou igual.</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v xml:space="preserve">  SOBRA   o que fazer com a fatia de um colocado em que ninguém apostou:</v>
+        <v xml:space="preserve">  Os percentuais não precisam somar 100: o bolo é dividido na proporção.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">          redividir (entre as outras faixas) ou clube.</v>
+        <v>A aba AJUSTES é opcional:</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  TAXA    % do bolo que fica com o clube antes da divisão.</v>
+        <v xml:space="preserve">  RATEIO  proporcional (quem apostou mais leva mais) ou igual.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">  SOBRA   o que fazer com a fatia de um colocado em que ninguém apostou:</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Depois é só importar em ⚙️ → Planilha → Importar planilha.</v>
+        <v xml:space="preserve">          redividir (entre as outras faixas) ou clube.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v xml:space="preserve">  TAXA    % do bolo que fica com o clube antes da divisão.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Depois é só importar em ⚙️ → Planilha → Importar planilha.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>Os nomes das abas e das colunas podem estar em qualquer ordem.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A37"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -734,8 +749,8 @@
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>200</v>
+      <c r="E2" t="str">
+        <v>bancou tudo</v>
       </c>
       <c r="F2" t="str">
         <v>cotas</v>

</xml_diff>